<commit_message>
after trying everything, final and last version of results
</commit_message>
<xml_diff>
--- a/goldStandard/_Assessment.xlsx
+++ b/goldStandard/_Assessment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia\Documents\GitHub\normScore\goldStandard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A55FD164-E9C3-4F72-96B8-A3A10797309D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9EBEAB2-2AC5-47AF-A9C3-A62F36BDB223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="19365" windowHeight="15240" xr2:uid="{47C0CA8E-5BD4-46FF-B103-6FF28F611458}"/>
+    <workbookView xWindow="420" yWindow="0" windowWidth="21195" windowHeight="20985" xr2:uid="{47C0CA8E-5BD4-46FF-B103-6FF28F611458}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1666" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1663" uniqueCount="170">
   <si>
     <t>Number</t>
   </si>
@@ -442,9 +442,6 @@
     <t>Quantile;VSN;CyclicLoess</t>
   </si>
   <si>
-    <t>Median;Log</t>
-  </si>
-  <si>
     <t>CyclicLoess;RLR</t>
   </si>
   <si>
@@ -521,9 +518,6 @@
     <t>Log;Median;Mean;TI</t>
   </si>
   <si>
-    <t>RLR;CyclicLoess</t>
-  </si>
-  <si>
     <t>Mean;TI;Log;Median</t>
   </si>
   <si>
@@ -546,6 +540,12 @@
   </si>
   <si>
     <t>Mean;CyclicLoess</t>
+  </si>
+  <si>
+    <t>Median;VSN;Quantile</t>
+  </si>
+  <si>
+    <t>Quantile;Log</t>
   </si>
 </sst>
 </file>
@@ -1212,13 +1212,13 @@
         <v>102</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>103</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J1" s="13" t="s">
         <v>109</v>
@@ -1240,7 +1240,7 @@
       <c r="A2" s="2"/>
       <c r="B2" s="17"/>
       <c r="C2" s="42" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>104</v>
@@ -1305,7 +1305,7 @@
         <v>Quantile</v>
       </c>
       <c r="J3" s="25" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K3" s="24" t="s">
         <v>112</v>
@@ -1455,7 +1455,7 @@
         <v>Quantile</v>
       </c>
       <c r="J6" s="26" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K6" s="30"/>
       <c r="L6" s="26">
@@ -1506,7 +1506,7 @@
         <v>116</v>
       </c>
       <c r="K7" s="30" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L7" s="26">
         <v>1</v>
@@ -1603,7 +1603,7 @@
         <v>Median</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="K9" s="3"/>
       <c r="L9" s="8">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="E10" t="str">
         <f>Item2!K9</f>
-        <v>CyclicLoess</v>
+        <v>Log</v>
       </c>
       <c r="F10" t="str">
         <f>Item3!K9</f>
@@ -1748,7 +1748,7 @@
         <v>Quantile</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K12" s="3" t="s">
         <v>112</v>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="E15" s="27" t="str">
         <f>Item2!K14</f>
-        <v>Log</v>
+        <v>CyclicLoess</v>
       </c>
       <c r="F15" s="27" t="str">
         <f>Item3!K14</f>
@@ -1942,7 +1942,7 @@
         <v>Quantile</v>
       </c>
       <c r="J16" s="26" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="K16" s="30" t="s">
         <v>112</v>
@@ -1989,10 +1989,10 @@
         <v>Quantile</v>
       </c>
       <c r="J17" s="26" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K17" s="30" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L17" s="26">
         <v>3</v>
@@ -2036,7 +2036,7 @@
         <v>Median</v>
       </c>
       <c r="J18" s="26" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K18" s="30" t="s">
         <v>131</v>
@@ -2083,10 +2083,10 @@
         <v>Quantile</v>
       </c>
       <c r="J19" s="26" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="K19" s="30" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L19" s="26">
         <v>3</v>
@@ -2180,7 +2180,7 @@
         <v>130</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L21" s="8">
         <v>4</v>
@@ -2269,7 +2269,7 @@
         <v>Quantile</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K23" s="3" t="s">
         <v>112</v>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="E24" t="str">
         <f>Item2!K23</f>
-        <v>Log</v>
+        <v>CyclicLoess</v>
       </c>
       <c r="F24" t="str">
         <f>Item3!K23</f>
@@ -2319,7 +2319,7 @@
         <v>116</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L24" s="8">
         <v>4</v>
@@ -2363,7 +2363,7 @@
         <v>CyclicLoess</v>
       </c>
       <c r="J25" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K25" s="3" t="s">
         <v>112</v>
@@ -2413,7 +2413,7 @@
         <v>116</v>
       </c>
       <c r="K26" s="30" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L26" s="26">
         <v>5</v>
@@ -2831,10 +2831,10 @@
         <v>RLR</v>
       </c>
       <c r="J35" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L35" s="8">
         <v>6</v>
@@ -3019,10 +3019,10 @@
         <v>Quantile</v>
       </c>
       <c r="J39" s="26" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K39" s="30" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L39" s="26">
         <v>7</v>
@@ -3113,10 +3113,10 @@
         <v>Median</v>
       </c>
       <c r="J41" s="26" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K41" s="30" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L41" s="26">
         <v>7</v>
@@ -3160,7 +3160,7 @@
         <v>Quantile</v>
       </c>
       <c r="J42" s="26" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="K42" s="30" t="s">
         <v>112</v>
@@ -3254,7 +3254,7 @@
         <v>Quantile</v>
       </c>
       <c r="J44" s="8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="K44" s="3" t="s">
         <v>112</v>
@@ -3393,7 +3393,7 @@
         <v>Quantile</v>
       </c>
       <c r="J47" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K47" s="3"/>
       <c r="L47" s="8">
@@ -3483,10 +3483,10 @@
         <v>Quantile</v>
       </c>
       <c r="J49" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="K49" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="L49" s="8">
         <v>8</v>
@@ -3530,7 +3530,7 @@
         <v>Quantile</v>
       </c>
       <c r="J50" s="26" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K50" s="30" t="s">
         <v>112</v>
@@ -3625,7 +3625,7 @@
         <v>116</v>
       </c>
       <c r="K52" s="30" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L52" s="26">
         <v>9</v>
@@ -3669,7 +3669,7 @@
         <v>Quantile</v>
       </c>
       <c r="J53" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K53" s="21" t="s">
         <v>131</v>
@@ -3716,7 +3716,7 @@
         <v>Quantile</v>
       </c>
       <c r="J54" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K54" s="8" t="s">
         <v>131</v>
@@ -3766,7 +3766,7 @@
         <v>132</v>
       </c>
       <c r="K55" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L55">
         <v>1</v>
@@ -3870,7 +3870,7 @@
         <v>27</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C58" t="s">
         <v>123</v>
@@ -4014,7 +4014,7 @@
       </c>
       <c r="D61" s="30" t="str">
         <f>Item1!K60</f>
-        <v>VSN</v>
+        <v>Log</v>
       </c>
       <c r="E61" s="27" t="str">
         <f>Item2!K60</f>
@@ -4022,7 +4022,7 @@
       </c>
       <c r="F61" s="27" t="str">
         <f>Item3!K60</f>
-        <v>VSN</v>
+        <v>CyclicLoess</v>
       </c>
       <c r="G61" s="27" t="str">
         <f>Item4!K60</f>
@@ -4030,18 +4030,16 @@
       </c>
       <c r="H61" s="27" t="str">
         <f>Item5!K60</f>
-        <v>VSN</v>
+        <v>Quantile</v>
       </c>
       <c r="I61" s="28" t="str">
         <f>Item6!K60</f>
-        <v>VSN</v>
+        <v>Quantile</v>
       </c>
       <c r="J61" s="27" t="s">
-        <v>118</v>
-      </c>
-      <c r="K61" s="26" t="s">
-        <v>161</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="K61" s="26"/>
       <c r="L61" s="27">
         <v>2</v>
       </c>
@@ -4129,7 +4127,7 @@
         <v>Quantile</v>
       </c>
       <c r="J63" s="27" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K63" s="26" t="s">
         <v>131</v>
@@ -4375,7 +4373,7 @@
         <v>23</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C69" t="s">
         <v>123</v>
@@ -4683,7 +4681,7 @@
         <v>Quantile</v>
       </c>
       <c r="J75" s="27" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K75" s="8"/>
       <c r="L75" s="27">
@@ -4728,10 +4726,10 @@
         <v>Quantile</v>
       </c>
       <c r="J76" t="s">
+        <v>168</v>
+      </c>
+      <c r="K76" s="8" t="s">
         <v>135</v>
-      </c>
-      <c r="K76" s="8" t="s">
-        <v>136</v>
       </c>
       <c r="L76">
         <v>5</v>
@@ -4778,7 +4776,7 @@
         <v>117</v>
       </c>
       <c r="K77" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="L77">
         <v>5</v>
@@ -4822,7 +4820,7 @@
         <v>Quantile</v>
       </c>
       <c r="J78" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="K78" s="8" t="s">
         <v>131</v>
@@ -4919,7 +4917,7 @@
         <v>132</v>
       </c>
       <c r="K80" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L80">
         <v>5</v>
@@ -4966,7 +4964,7 @@
         <v>116</v>
       </c>
       <c r="K81" s="8" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="L81">
         <v>5</v>
@@ -5100,7 +5098,7 @@
         <v>Quantile</v>
       </c>
       <c r="J84" s="27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K84" s="26"/>
       <c r="L84" s="27">
@@ -5190,10 +5188,10 @@
         <v>Quantile</v>
       </c>
       <c r="J86" s="27" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="K86" s="26" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L86" s="27">
         <v>6</v>
@@ -5218,7 +5216,7 @@
       </c>
       <c r="E87" s="27" t="str">
         <f>Item2!K86</f>
-        <v>Log</v>
+        <v>CyclicLoess</v>
       </c>
       <c r="F87" s="27" t="str">
         <f>Item3!K86</f>
@@ -5284,7 +5282,7 @@
         <v>Median</v>
       </c>
       <c r="J88" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="K88" s="8"/>
       <c r="L88">
@@ -5331,9 +5329,7 @@
       <c r="J89" t="s">
         <v>133</v>
       </c>
-      <c r="K89" s="8" t="s">
-        <v>112</v>
-      </c>
+      <c r="K89" s="8"/>
       <c r="L89">
         <v>7</v>
       </c>
@@ -5468,9 +5464,7 @@
       <c r="J92" t="s">
         <v>114</v>
       </c>
-      <c r="K92" s="8" t="s">
-        <v>158</v>
-      </c>
+      <c r="K92" s="8"/>
       <c r="L92">
         <v>7</v>
       </c>
@@ -5494,7 +5488,7 @@
       </c>
       <c r="E93" t="str">
         <f>Item2!K92</f>
-        <v>Log</v>
+        <v>CyclicLoess</v>
       </c>
       <c r="F93" t="str">
         <f>Item3!K92</f>
@@ -5648,7 +5642,7 @@
         <v>Quantile</v>
       </c>
       <c r="J96" s="27" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="K96" s="26" t="s">
         <v>132</v>
@@ -5742,7 +5736,7 @@
         <v>Quantile</v>
       </c>
       <c r="J98" s="27" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K98" s="26"/>
       <c r="L98" s="27">
@@ -5880,7 +5874,7 @@
         <v>132</v>
       </c>
       <c r="K101" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L101">
         <v>9</v>
@@ -5940,6 +5934,7 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7926,7 +7921,7 @@
         <v>27</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C57" s="3">
         <v>6</v>
@@ -8034,16 +8029,16 @@
         <v>57</v>
       </c>
       <c r="C60" s="30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D60" s="27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E60" s="27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60" s="27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G60" s="27">
         <v>3</v>
@@ -8052,13 +8047,13 @@
         <v>5</v>
       </c>
       <c r="I60" s="27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J60" s="28">
         <v>4</v>
       </c>
       <c r="K60" s="28" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
@@ -8311,7 +8306,7 @@
         <v>23</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C68" s="3">
         <v>6</v>
@@ -9807,31 +9802,31 @@
         <v>7</v>
       </c>
       <c r="C9" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -9982,31 +9977,31 @@
         <v>78</v>
       </c>
       <c r="C14" s="30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" s="27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" s="27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" s="27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H14" s="27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I14" s="27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J14" s="28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" s="28" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -10297,31 +10292,31 @@
         <v>40</v>
       </c>
       <c r="C23" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J23" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -11484,7 +11479,7 @@
         <v>27</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C57" s="3">
         <v>2</v>
@@ -11869,7 +11864,7 @@
         <v>23</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C68" s="3">
         <v>2</v>
@@ -12502,31 +12497,31 @@
         <v>68</v>
       </c>
       <c r="C86" s="30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D86" s="27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E86" s="27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F86" s="27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G86" s="27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H86" s="27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I86" s="27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J86" s="28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K86" s="28" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
@@ -12712,31 +12707,31 @@
         <v>34</v>
       </c>
       <c r="C92" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D92">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E92">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F92">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G92">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H92">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I92">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J92" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K92" s="4" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.25">
@@ -15042,7 +15037,7 @@
         <v>27</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C57" s="3">
         <v>3</v>
@@ -15165,16 +15160,16 @@
         <v>4</v>
       </c>
       <c r="H60" s="27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I60" s="27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J60" s="28">
         <v>5</v>
       </c>
       <c r="K60" s="28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
@@ -15401,7 +15396,7 @@
         <v>1</v>
       </c>
       <c r="E67">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F67">
         <v>1</v>
@@ -15410,7 +15405,7 @@
         <v>1</v>
       </c>
       <c r="H67">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I67">
         <v>2</v>
@@ -15427,7 +15422,7 @@
         <v>23</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C68" s="3">
         <v>3</v>
@@ -18601,7 +18596,7 @@
         <v>27</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C57" s="3">
         <v>3</v>
@@ -18986,7 +18981,7 @@
         <v>23</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C68" s="3">
         <v>3</v>
@@ -22159,7 +22154,7 @@
         <v>27</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C57" s="3">
         <v>1</v>
@@ -22270,28 +22265,28 @@
         <v>2</v>
       </c>
       <c r="D60" s="27">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E60" s="27">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F60" s="27">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G60" s="27">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H60" s="27">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I60" s="27">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J60" s="28">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K60" s="28" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
@@ -22544,7 +22539,7 @@
         <v>23</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C68" s="3">
         <v>1</v>
@@ -25717,7 +25712,7 @@
         <v>27</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C57" s="3">
         <v>3</v>
@@ -25825,7 +25820,7 @@
         <v>57</v>
       </c>
       <c r="C60" s="30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D60" s="27">
         <v>2</v>
@@ -25837,19 +25832,19 @@
         <v>2</v>
       </c>
       <c r="G60" s="27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H60" s="27">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I60" s="27">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J60" s="28">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K60" s="28" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
@@ -26102,7 +26097,7 @@
         <v>23</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C68" s="3">
         <v>3</v>

</xml_diff>